<commit_message>
Master Matchmakers deck: re-sequenced plan largest-to-smallest metro + LGBTQ article removed
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
@@ -1809,38 +1809,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Matchmaking for Gay Singles in Los Angeles</t>
+          <t>Where Los Angeles Professionals Actually Meet Someone</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>gay matchmaker los angeles</t>
+          <t>los angeles dating scene</t>
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>110</v>
+        <v>700</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>City Matchmaker Pages</t>
+        <v>25</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Local Dating Guides</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>KD 3. Niche-local page, near-zero difficulty.</t>
+          <t>LA dating-scene support blog; links up to the LA location page.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
@@ -2579,7 +2579,7 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
@@ -3216,7 +3216,7 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
@@ -3706,7 +3706,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="J67" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K67" s="7" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K82" s="7" t="inlineStr">
         <is>
@@ -4784,7 +4784,7 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K86" s="7" t="inlineStr">
         <is>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="J91" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K91" s="7" t="inlineStr">
         <is>
@@ -5078,7 +5078,7 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K92" s="7" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K98" s="7" t="inlineStr">
         <is>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="J99" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K99" s="7" t="inlineStr">
         <is>
@@ -20727,28 +20727,28 @@
     <row r="431">
       <c r="A431" s="3" t="inlineStr">
         <is>
-          <t>gay matchmaker los angeles</t>
+          <t>los angeles dating scene</t>
         </is>
       </c>
       <c r="B431" s="4" t="n">
-        <v>110</v>
+        <v>700</v>
       </c>
       <c r="C431" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D431" s="5" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="E431" s="11" t="inlineStr">
-        <is>
-          <t>City Matchmaker Pages</t>
+        <v>25</v>
+      </c>
+      <c r="D431" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E431" s="10" t="inlineStr">
+        <is>
+          <t>Local Dating Guides</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="G431" s="15" t="inlineStr">
@@ -23449,7 +23449,7 @@
     <row r="14" ht="66" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  City Matchmaker Pages   — your localization money pages: '[city] matchmaker' for metros you don't have a page for yet, plus niche-local (Jewish/gay/elite). This is the direct answer to Luma's local-page strategy.
+          <t xml:space="preserve">  City Matchmaker Pages   — your localization money pages: '[city] matchmaker' for metros you don't have a page for yet, plus niche-local (Jewish/elite/luxury). This is the direct answer to Luma's local-page strategy.
   Local Dating Guides     — 'date ideas / date night [city]' — low-difficulty local content that wins AI overviews and feeds your city pages. These are the exact terms Luma already ranks for and you don't.
   Matchmaking 101 &amp; Cost  — the buyer-decision questions ('how much does a matchmaker cost', 'are matchmakers worth it') that AI engines answer directly. Owning these puts you in the AI answer for someone choosing a matchmaker.
   Dating Coaching         — first-date, life-stage and relationship advice that builds topical authority and captures the app-fatigued searcher before they're ready to hire.</t>
@@ -23467,9 +23467,9 @@
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  120 articles, split exactly 40/40/40 across Months 1-3
-  76,560 total monthly searches addressed
+  77,150 total monthly searches addressed
   96 easy wins at KD &lt; 30 — front-loaded into Month 1 so you see local rankings early
-  Average difficulty KD 19.8 — deliberately achievable, weighted toward winnable local terms</t>
+  Average difficulty KD 20.0 — deliberately achievable, weighted toward winnable local terms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master Matchmakers deck: varied article titles (no more repeated 'Find a Matchmaker in X')
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in New York</t>
+          <t>New York Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Date Ideas in New York Worth Leaving the House For</t>
+          <t>New York Date Ideas Locals Actually Love</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Los Angeles</t>
+          <t>Looking for a Matchmaker in Los Angeles?</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Date Ideas in Los Angeles Worth Leaving the House For</t>
+          <t>Where to Take a Date in Los Angeles</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Date Night in Los Angeles: A Local Guide</t>
+          <t>Los Angeles Date Nights That Actually Impress</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Los Angeles</t>
+          <t>Los Angeles Dating, With Expert Coaching</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Chicago</t>
+          <t>Meet Your Match in Chicago</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Date Ideas in Chicago Worth Leaving the House For</t>
+          <t>The Best Date Ideas in Chicago</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Date Night in Chicago: A Local Guide</t>
+          <t>Romantic Date Nights in Chicago</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Chicago</t>
+          <t>The Chicago Dating Scene for Busy Professionals</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Chicago</t>
+          <t>How to Date Smarter in Chicago</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Dallas</t>
+          <t>How to Find a Great Matchmaker in Dallas</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Date Ideas in Dallas Worth Leaving the House For</t>
+          <t>Creative Date Ideas in Dallas</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Date Night in Dallas: A Local Guide</t>
+          <t>The Dallas Date-Night Playbook</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Dallas</t>
+          <t>How to Meet Someone in Dallas Without Swiping</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Dallas</t>
+          <t>Dating Coaching for Dallas Professionals</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Houston</t>
+          <t>Why Houston Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Date Ideas in Houston Worth Leaving the House For</t>
+          <t>Houston Date Ideas, From First Date to Fifth</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Date Night in Houston: A Local Guide</t>
+          <t>Where to Spend Date Night in Houston</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Houston</t>
+          <t>Where Houston Professionals Actually Meet</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Houston</t>
+          <t>Making Time to Date in Houston</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Washington</t>
+          <t>Your Personal Matchmaker in Washington</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Date Ideas in Washington Worth Leaving the House For</t>
+          <t>Date Ideas in Washington Beyond Dinner and a Movie</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Date Night in Washington: A Local Guide</t>
+          <t>Date Night Done Right in Washington</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Washington</t>
+          <t>A Smarter Approach to Dating in Washington</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Philadelphia</t>
+          <t>Professional Matchmaking in Philadelphia, Explained</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Date Ideas in Philadelphia Worth Leaving the House For</t>
+          <t>Fresh Date Ideas Worth Trying in Philadelphia</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Date Night in Philadelphia: A Local Guide</t>
+          <t>Philadelphia After Dark: Date-Night Ideas</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Atlanta</t>
+          <t>Is Hiring a Matchmaker Worth It in Atlanta?</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Date Ideas in Atlanta Worth Leaving the House For</t>
+          <t>Memorable Date Ideas Around Atlanta</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Date Night in Atlanta: A Local Guide</t>
+          <t>Planning the Perfect Atlanta Date Night</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Atlanta</t>
+          <t>Meeting Quality Singles in Atlanta</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Atlanta</t>
+          <t>Dating Confidently in Atlanta</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Miami</t>
+          <t>The Modern Way to Date in Miami</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Date Ideas in Miami Worth Leaving the House For</t>
+          <t>Miami Date Ideas Locals Actually Love</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Miami</t>
+          <t>Miami Dating Tips From the Experts</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Phoenix</t>
+          <t>Hand-Picked Introductions for Phoenix Singles</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Date Ideas in Phoenix Worth Leaving the House For</t>
+          <t>Where to Take a Date in Phoenix</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Date Night in Phoenix: A Local Guide</t>
+          <t>Phoenix Date Nights That Actually Impress</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Boston</t>
+          <t>Matchmaking in Boston for Busy Professionals</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Date Ideas in Boston Worth Leaving the House For</t>
+          <t>The Best Date Ideas in Boston</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Date Night in Boston: A Local Guide</t>
+          <t>Romantic Date Nights in Boston</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Boston</t>
+          <t>The Best Places to Meet Singles in Boston</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Boston</t>
+          <t>Boston Dating, With Expert Coaching</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in San Francisco</t>
+          <t>What a San Francisco Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Date Ideas in San Francisco Worth Leaving the House For</t>
+          <t>Creative Date Ideas in San Francisco</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Date Night in San Francisco: A Local Guide</t>
+          <t>The San Francisco Date-Night Playbook</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in San Francisco</t>
+          <t>How to Date Smarter in San Francisco</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Detroit</t>
+          <t>Serious About Dating in Detroit? Consider a Matchmaker</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Seattle</t>
+          <t>Seattle's Alternative to Endless Swiping</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3328,7 +3328,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Date Ideas in Seattle Worth Leaving the House For</t>
+          <t>Seattle Date Ideas, From First Date to Fifth</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Date Night in Seattle: A Local Guide</t>
+          <t>Where to Spend Date Night in Seattle</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Seattle</t>
+          <t>Dating in Seattle: Where to Actually Meet People</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Minneapolis</t>
+          <t>Finding Love in Minneapolis, the Personal Way</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Date Ideas in Minneapolis Worth Leaving the House For</t>
+          <t>Date Ideas in Minneapolis Beyond Dinner and a Movie</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in San Diego</t>
+          <t>San Diego Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Date Ideas in San Diego Worth Leaving the House For</t>
+          <t>Fresh Date Ideas Worth Trying in San Diego</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in San Diego</t>
+          <t>How Professionals Find Their Match in San Diego</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in San Diego</t>
+          <t>Dating Coaching for San Diego Professionals</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Tampa</t>
+          <t>Looking for a Matchmaker in Tampa?</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Date Ideas in Tampa Worth Leaving the House For</t>
+          <t>Memorable Date Ideas Around Tampa</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Date Night in Tampa: A Local Guide</t>
+          <t>Date Night Done Right in Tampa</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Tampa</t>
+          <t>Making Time to Date in Tampa</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Denver</t>
+          <t>Meet Your Match in Denver</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Date Ideas in Denver Worth Leaving the House For</t>
+          <t>Denver Date Ideas Locals Actually Love</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Date Night in Denver: A Local Guide</t>
+          <t>Denver After Dark: Date-Night Ideas</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Denver</t>
+          <t>The Denver Dating Scene for Busy Professionals</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Denver</t>
+          <t>A Smarter Approach to Dating in Denver</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Baltimore</t>
+          <t>How to Find a Great Matchmaker in Baltimore</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Date Ideas in Baltimore Worth Leaving the House For</t>
+          <t>Where to Take a Date in Baltimore</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4357,7 +4357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Date Night in Baltimore: A Local Guide</t>
+          <t>Planning the Perfect Baltimore Date Night</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Baltimore</t>
+          <t>Dating Confidently in Baltimore</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in St. Louis</t>
+          <t>Why St. Louis Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Date Ideas in St. Louis Worth Leaving the House For</t>
+          <t>The Best Date Ideas in St. Louis</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in St. Louis</t>
+          <t>St. Louis Dating Tips From the Experts</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Charlotte</t>
+          <t>Your Personal Matchmaker in Charlotte</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Charlotte</t>
+          <t>How to Meet Someone in Charlotte Without Swiping</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Orlando</t>
+          <t>Professional Matchmaking in Orlando, Explained</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Date Ideas in Orlando Worth Leaving the House For</t>
+          <t>Creative Date Ideas in Orlando</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Date Night in Orlando: A Local Guide</t>
+          <t>Orlando Date Nights That Actually Impress</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in San Antonio</t>
+          <t>Is Hiring a Matchmaker Worth It in San Antonio?</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Portland</t>
+          <t>The Modern Way to Date in Portland</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Sacramento</t>
+          <t>Hand-Picked Introductions for Sacramento Singles</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Pittsburgh</t>
+          <t>Matchmaking in Pittsburgh for Busy Professionals</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Las Vegas</t>
+          <t>What a Las Vegas Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Cincinnati</t>
+          <t>Serious About Dating in Cincinnati? Consider a Matchmaker</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Kansas City</t>
+          <t>Kansas City's Alternative to Endless Swiping</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Columbus</t>
+          <t>Finding Love in Columbus, the Personal Way</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Cleveland</t>
+          <t>Cleveland Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Indianapolis</t>
+          <t>Looking for a Matchmaker in Indianapolis?</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Nashville</t>
+          <t>Meet Your Match in Nashville</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Milwaukee</t>
+          <t>How to Find a Great Matchmaker in Milwaukee</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Jacksonville</t>
+          <t>Why Jacksonville Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Oklahoma City</t>
+          <t>Your Personal Matchmaker in Oklahoma City</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Raleigh</t>
+          <t>Professional Matchmaking in Raleigh, Explained</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Memphis</t>
+          <t>Is Hiring a Matchmaker Worth It in Memphis?</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Richmond</t>
+          <t>The Modern Way to Date in Richmond</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in New Orleans</t>
+          <t>Hand-Picked Introductions for New Orleans Singles</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Louisville</t>
+          <t>Matchmaking in Louisville for Busy Professionals</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Buffalo</t>
+          <t>What a Buffalo Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Salt Lake City</t>
+          <t>Serious About Dating in Salt Lake City? Consider a Matchmaker</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Birmingham</t>
+          <t>Birmingham's Alternative to Endless Swiping</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Tucson</t>
+          <t>Finding Love in Tucson, the Personal Way</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Tulsa</t>
+          <t>Tulsa Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Omaha</t>
+          <t>Looking for a Matchmaker in Omaha?</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Albuquerque</t>
+          <t>Meet Your Match in Albuquerque</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Knoxville</t>
+          <t>How to Find a Great Matchmaker in Knoxville</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Boise</t>
+          <t>Why Boise Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Des Moines</t>
+          <t>Your Personal Matchmaker in Des Moines</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Spokane</t>
+          <t>Professional Matchmaking in Spokane, Explained</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -6415,7 +6415,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Reno</t>
+          <t>Is Hiring a Matchmaker Worth It in Reno?</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Find a Matchmaker in Naples</t>
+          <t>The Modern Way to Date in Naples</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Master Matchmakers deck: keyword-in-title money pages + a/an fix
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Meet Your Match in Chicago</t>
+          <t>How to Find a Great Matchmaker in Chicago</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Dallas</t>
+          <t>Why Dallas Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Why Houston Singles Are Turning to Matchmakers</t>
+          <t>Professional Matchmaking in Houston, Explained</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Washington</t>
+          <t>Is Hiring a Matchmaker Worth It in Washington?</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Philadelphia, Explained</t>
+          <t>Matchmaking in Philadelphia for Busy Professionals</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Atlanta?</t>
+          <t>What an Atlanta Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>The Modern Way to Date in Miami</t>
+          <t>Your Personal Matchmaker in Miami</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hand-Picked Introductions for Phoenix Singles</t>
+          <t>Phoenix Matchmaking, Done for You</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Matchmaking in Boston for Busy Professionals</t>
+          <t>Meet Your Match With a Boston Matchmaker</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>What a San Francisco Matchmaker Actually Does</t>
+          <t>The San Francisco Matchmaker for Serious Singles</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Serious About Dating in Detroit? Consider a Matchmaker</t>
+          <t>Serious About Dating in Detroit? Meet a Matchmaker</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Seattle's Alternative to Endless Swiping</t>
+          <t>Finding Love in Seattle With a Matchmaker</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Finding Love in Minneapolis, the Personal Way</t>
+          <t>A Minneapolis Matchmaker's Take on Modern Dating</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Meet Your Match in Denver</t>
+          <t>How to Find a Great Matchmaker in Denver</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Baltimore</t>
+          <t>Why Baltimore Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Why St. Louis Singles Are Turning to Matchmakers</t>
+          <t>Professional Matchmaking in St. Louis, Explained</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Charlotte</t>
+          <t>Is Hiring a Matchmaker Worth It in Charlotte?</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Orlando, Explained</t>
+          <t>Matchmaking in Orlando for Busy Professionals</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in San Antonio?</t>
+          <t>What a San Antonio Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>The Modern Way to Date in Portland</t>
+          <t>Your Personal Matchmaker in Portland</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Hand-Picked Introductions for Sacramento Singles</t>
+          <t>Sacramento Matchmaking, Done for You</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Matchmaking in Pittsburgh for Busy Professionals</t>
+          <t>Meet Your Match With a Pittsburgh Matchmaker</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>What a Las Vegas Matchmaker Actually Does</t>
+          <t>The Las Vegas Matchmaker for Serious Singles</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Serious About Dating in Cincinnati? Consider a Matchmaker</t>
+          <t>Serious About Dating in Cincinnati? Meet a Matchmaker</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Kansas City's Alternative to Endless Swiping</t>
+          <t>Finding Love in Kansas City With a Matchmaker</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Finding Love in Columbus, the Personal Way</t>
+          <t>A Columbus Matchmaker's Take on Modern Dating</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Meet Your Match in Nashville</t>
+          <t>How to Find a Great Matchmaker in Nashville</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Milwaukee</t>
+          <t>Why Milwaukee Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Why Jacksonville Singles Are Turning to Matchmakers</t>
+          <t>Professional Matchmaking in Jacksonville, Explained</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Oklahoma City</t>
+          <t>Is Hiring a Matchmaker Worth It in Oklahoma City?</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Raleigh, Explained</t>
+          <t>Matchmaking in Raleigh for Busy Professionals</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Memphis?</t>
+          <t>What a Memphis Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>The Modern Way to Date in Richmond</t>
+          <t>Your Personal Matchmaker in Richmond</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Hand-Picked Introductions for New Orleans Singles</t>
+          <t>New Orleans Matchmaking, Done for You</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Matchmaking in Louisville for Busy Professionals</t>
+          <t>Meet Your Match With a Louisville Matchmaker</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>What a Buffalo Matchmaker Actually Does</t>
+          <t>The Buffalo Matchmaker for Serious Singles</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Serious About Dating in Salt Lake City? Consider a Matchmaker</t>
+          <t>Serious About Dating in Salt Lake City? Meet a Matchmaker</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Birmingham's Alternative to Endless Swiping</t>
+          <t>Finding Love in Birmingham With a Matchmaker</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Finding Love in Tucson, the Personal Way</t>
+          <t>A Tucson Matchmaker's Take on Modern Dating</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Meet Your Match in Albuquerque</t>
+          <t>How to Find a Great Matchmaker in Albuquerque</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Knoxville</t>
+          <t>Why Knoxville Singles Are Turning to Matchmakers</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Why Boise Singles Are Turning to Matchmakers</t>
+          <t>Professional Matchmaking in Boise, Explained</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Des Moines</t>
+          <t>Is Hiring a Matchmaker Worth It in Des Moines?</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Spokane, Explained</t>
+          <t>Matchmaking in Spokane for Busy Professionals</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -6415,7 +6415,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Reno?</t>
+          <t>What a Reno Matchmaker Actually Does</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>The Modern Way to Date in Naples</t>
+          <t>Your Personal Matchmaker in Naples</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">

</xml_diff>

<commit_message>
MM deck: SEO-length titles (~50-60 chars)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -682,7 +682,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New York Date Ideas Locals Actually Love</t>
+          <t>New York Date Ideas Locals Actually Love, Season by Season</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Date Night in New York: A Local Guide</t>
+          <t>Date Night in New York: A Local Guide to the Best Spots</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in New York</t>
+          <t>Dating for Busy Professionals in New York: Make Time for Love</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Los Angeles?</t>
+          <t>Looking for a Matchmaker in Los Angeles? Here's How to Choose</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Where to Take a Date in Los Angeles</t>
+          <t>Where to Take a Date in Los Angeles: A Local's Shortlist</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Los Angeles Date Nights That Actually Impress</t>
+          <t>Los Angeles Date Nights That Actually Impress a Date</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Los Angeles</t>
+          <t>Where to Meet Singles in Los Angeles Without the Apps</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Los Angeles Dating, With Expert Coaching</t>
+          <t>Los Angeles Dating, With Expert Coaching That Actually Helps</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Chicago</t>
+          <t>How to Find a Matchmaker in Chicago You Can Actually Trust</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>The Best Date Ideas in Chicago</t>
+          <t>The Best Date Ideas in Chicago for Every Kind of Couple</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Romantic Date Nights in Chicago</t>
+          <t>Romantic Date Nights in Chicago for Every Season</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The Chicago Dating Scene for Busy Professionals</t>
+          <t>The Chicago Dating Scene for Busy Professionals, Decoded</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>How to Date Smarter in Chicago</t>
+          <t>How to Date Smarter in Chicago and Stop Wasting Time</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Why Dallas Singles Are Turning to Matchmakers</t>
+          <t>Why Dallas Singles Are Choosing Professional Matchmakers</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Creative Date Ideas in Dallas</t>
+          <t>Creative Date Ideas in Dallas Beyond Dinner and a Movie</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The Dallas Date-Night Playbook</t>
+          <t>The Dallas Date-Night Playbook, From Casual to Elegant</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>How to Meet Someone in Dallas Without Swiping</t>
+          <t>How to Meet Someone in Dallas When Swiping Isn't Working</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dating Coaching for Dallas Professionals</t>
+          <t>Dating Coaching for Dallas Professionals Who Are Serious</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Houston, Explained</t>
+          <t>Professional Matchmaking in Houston: What to Expect</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Houston Date Ideas, From First Date to Fifth</t>
+          <t>Houston Date Ideas, From a Casual First Date to the Fifth</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Where to Spend Date Night in Houston</t>
+          <t>Where to Spend Date Night in Houston Without the Guesswork</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Where Houston Professionals Actually Meet</t>
+          <t>Where Houston Professionals Actually Meet Their Match</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Making Time to Date in Houston</t>
+          <t>Making Time to Date in Houston When Life Is Busy</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Washington?</t>
+          <t>Is Hiring a Matchmaker in Washington Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Date Ideas in Washington Beyond Dinner and a Movie</t>
+          <t>Date Ideas in Washington That Actually Lead Somewhere</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Date Night Done Right in Washington</t>
+          <t>Date Night Done Right in Washington: Ideas That Land</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>A Smarter Approach to Dating in Washington</t>
+          <t>A Smarter Approach to Dating in Washington for Professionals</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Matchmaking in Philadelphia for Busy Professionals</t>
+          <t>What a Philadelphia Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fresh Date Ideas Worth Trying in Philadelphia</t>
+          <t>Fresh Philadelphia Date Ideas Worth Leaving the House For</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Philadelphia After Dark: Date-Night Ideas</t>
+          <t>Philadelphia After Dark: Date-Night Ideas Worth Planning</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>What an Atlanta Matchmaker Actually Does</t>
+          <t>Your Personal Matchmaker in Atlanta: Introductions Done Right</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Memorable Date Ideas Around Atlanta</t>
+          <t>Memorable Date Ideas Around Atlanta for Any Budget</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Planning the Perfect Atlanta Date Night</t>
+          <t>Planning the Perfect Date Night in Atlanta</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Meeting Quality Singles in Atlanta</t>
+          <t>Meeting Quality Singles in Atlanta: A Practical Guide</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dating Confidently in Atlanta</t>
+          <t>Dating Confidently in Atlanta: Advice From the Experts</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Miami</t>
+          <t>Miami Matchmaking, Done for You From Vetting to First Date</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Miami Date Ideas Locals Actually Love</t>
+          <t>Miami Date Ideas Locals Actually Love, Season by Season</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Date Night in Miami: A Local Guide</t>
+          <t>Date Night in Miami: A Local Guide to the Best Spots</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Miami Dating Tips From the Experts</t>
+          <t>Miami Dating Tips From Professional Matchmakers</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Phoenix Matchmaking, Done for You</t>
+          <t>Meet Someone Worth Your Time With a Phoenix Matchmaker</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Where to Take a Date in Phoenix</t>
+          <t>Where to Take a Date in Phoenix: A Local's Shortlist</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Phoenix Date Nights That Actually Impress</t>
+          <t>Phoenix Date Nights That Actually Impress a Date</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Phoenix</t>
+          <t>Dating for Busy Professionals in Phoenix: Make Time for Love</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Meet Your Match With a Boston Matchmaker</t>
+          <t>The Boston Matchmaker for Marriage-Minded Professionals</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>The Best Date Ideas in Boston</t>
+          <t>The Best Date Ideas in Boston for Every Kind of Couple</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Romantic Date Nights in Boston</t>
+          <t>Romantic Date Nights in Boston for Every Season</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>The Best Places to Meet Singles in Boston</t>
+          <t>The Best Places to Meet Singles in Boston in Real Life</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Boston Dating, With Expert Coaching</t>
+          <t>Boston Dating, With Expert Coaching That Actually Helps</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The San Francisco Matchmaker for Serious Singles</t>
+          <t>Serious About Dating in San Francisco? A Matchmaker Can Help</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Creative Date Ideas in San Francisco</t>
+          <t>Creative Date Ideas in San Francisco Beyond Dinner and a Movie</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>The San Francisco Date-Night Playbook</t>
+          <t>The San Francisco Date-Night Playbook, From Casual to Elegant</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>How to Date Smarter in San Francisco</t>
+          <t>How to Date Smarter in San Francisco and Stop Wasting Time</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Serious About Dating in Detroit? Meet a Matchmaker</t>
+          <t>Finding Love in Detroit With a Professional Matchmaker</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Finding Love in Seattle With a Matchmaker</t>
+          <t>A Seattle Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3328,7 +3328,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Seattle Date Ideas, From First Date to Fifth</t>
+          <t>Seattle Date Ideas, From a Casual First Date to the Fifth</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Where to Spend Date Night in Seattle</t>
+          <t>Where to Spend Date Night in Seattle Without the Guesswork</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dating in Seattle: Where to Actually Meet People</t>
+          <t>Dating in Seattle: Where to Actually Meet Real People</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>A Minneapolis Matchmaker's Take on Modern Dating</t>
+          <t>Minneapolis Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Date Ideas in Minneapolis Beyond Dinner and a Movie</t>
+          <t>Date Ideas in Minneapolis That Actually Lead Somewhere</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>San Diego Matchmaker: How Personalized Matchmaking Works</t>
+          <t>Looking for a Matchmaker in San Diego? Here's How to Choose</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Fresh Date Ideas Worth Trying in San Diego</t>
+          <t>Fresh San Diego Date Ideas Worth Leaving the House For</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dating Coaching for San Diego Professionals</t>
+          <t>Dating Coaching for San Diego Professionals Who Are Serious</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Tampa?</t>
+          <t>How to Find a Matchmaker in Tampa You Can Actually Trust</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Memorable Date Ideas Around Tampa</t>
+          <t>Memorable Date Ideas Around Tampa for Any Budget</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Date Night Done Right in Tampa</t>
+          <t>Date Night Done Right in Tampa: Ideas That Land</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Where to Meet Singles in Tampa</t>
+          <t>Where to Meet Singles in Tampa Without the Apps</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Making Time to Date in Tampa</t>
+          <t>Making Time to Date in Tampa When Life Is Busy</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Denver</t>
+          <t>Why Denver Singles Are Choosing Professional Matchmakers</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Denver Date Ideas Locals Actually Love</t>
+          <t>Denver Date Ideas Locals Actually Love, Season by Season</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Denver After Dark: Date-Night Ideas</t>
+          <t>Denver After Dark: Date-Night Ideas Worth Planning</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>The Denver Dating Scene for Busy Professionals</t>
+          <t>The Denver Dating Scene for Busy Professionals, Decoded</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>A Smarter Approach to Dating in Denver</t>
+          <t>A Smarter Approach to Dating in Denver for Professionals</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Why Baltimore Singles Are Turning to Matchmakers</t>
+          <t>Professional Matchmaking in Baltimore: What to Expect</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Where to Take a Date in Baltimore</t>
+          <t>Where to Take a Date in Baltimore: A Local's Shortlist</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4357,7 +4357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Planning the Perfect Baltimore Date Night</t>
+          <t>Planning the Perfect Date Night in Baltimore</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dating Confidently in Baltimore</t>
+          <t>Dating Confidently in Baltimore: Advice From the Experts</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in St. Louis, Explained</t>
+          <t>Is Hiring a Matchmaker in St. Louis Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>The Best Date Ideas in St. Louis</t>
+          <t>The Best Date Ideas in St. Louis for Every Kind of Couple</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Date Night in St. Louis: A Local Guide</t>
+          <t>Date Night in St. Louis: A Local Guide to the Best Spots</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>St. Louis Dating Tips From the Experts</t>
+          <t>St. Louis Dating Tips From Professional Matchmakers</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Charlotte?</t>
+          <t>Matchmaking in Charlotte for Busy, Relationship-Ready Singles</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>How to Meet Someone in Charlotte Without Swiping</t>
+          <t>How to Meet Someone in Charlotte When Swiping Isn't Working</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Dating for Busy Professionals in Charlotte</t>
+          <t>Dating for Busy Professionals in Charlotte: Make Time for Love</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Matchmaking in Orlando for Busy Professionals</t>
+          <t>What an Orlando Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Creative Date Ideas in Orlando</t>
+          <t>Creative Date Ideas in Orlando Beyond Dinner and a Movie</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Orlando Date Nights That Actually Impress</t>
+          <t>Orlando Date Nights That Actually Impress a Date</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>What a San Antonio Matchmaker Actually Does</t>
+          <t>Meet Someone Worth Your Time With a San Antonio Matchmaker</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Portland</t>
+          <t>The Portland Matchmaker for Marriage-Minded Professionals</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Sacramento Matchmaking, Done for You</t>
+          <t>Serious About Dating in Sacramento? A Matchmaker Can Help</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Meet Your Match With a Pittsburgh Matchmaker</t>
+          <t>Finding Love in Pittsburgh With a Professional Matchmaker</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>The Las Vegas Matchmaker for Serious Singles</t>
+          <t>A Las Vegas Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Serious About Dating in Cincinnati? Meet a Matchmaker</t>
+          <t>Cincinnati Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Finding Love in Kansas City With a Matchmaker</t>
+          <t>Looking for a Matchmaker in Kansas City? Here's How to Choose</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>A Columbus Matchmaker's Take on Modern Dating</t>
+          <t>How to Find a Matchmaker in Columbus You Can Actually Trust</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Cleveland Matchmaker: How Personalized Matchmaking Works</t>
+          <t>Why Cleveland Singles Are Choosing Professional Matchmakers</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Indianapolis?</t>
+          <t>Professional Matchmaking in Indianapolis: What to Expect</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Nashville</t>
+          <t>Is Hiring a Matchmaker in Nashville Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Why Milwaukee Singles Are Turning to Matchmakers</t>
+          <t>Matchmaking in Milwaukee for Busy, Relationship-Ready Singles</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Jacksonville, Explained</t>
+          <t>What a Jacksonville Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Oklahoma City?</t>
+          <t>Meet Someone Worth Your Time With an Oklahoma City Matchmaker</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Matchmaking in Raleigh for Busy Professionals</t>
+          <t>The Raleigh Matchmaker for Marriage-Minded Professionals</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>What a Memphis Matchmaker Actually Does</t>
+          <t>Serious About Dating in Memphis? A Matchmaker Can Help</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Richmond</t>
+          <t>Finding Love in Richmond With a Professional Matchmaker</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>New Orleans Matchmaking, Done for You</t>
+          <t>A New Orleans Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Meet Your Match With a Louisville Matchmaker</t>
+          <t>Louisville Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>The Buffalo Matchmaker for Serious Singles</t>
+          <t>Looking for a Matchmaker in Buffalo? Here's How to Choose</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Serious About Dating in Salt Lake City? Meet a Matchmaker</t>
+          <t>Professional Matchmaking in Salt Lake City: What to Expect</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Finding Love in Birmingham With a Matchmaker</t>
+          <t>Is Hiring a Matchmaker in Birmingham Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>A Tucson Matchmaker's Take on Modern Dating</t>
+          <t>Matchmaking in Tucson for Busy, Relationship-Ready Singles</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Tulsa Matchmaker: How Personalized Matchmaking Works</t>
+          <t>What a Tulsa Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Omaha?</t>
+          <t>Your Personal Matchmaker in Omaha: Introductions Done Right</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>How to Find a Great Matchmaker in Albuquerque</t>
+          <t>Meet Someone Worth Your Time With an Albuquerque Matchmaker</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Why Knoxville Singles Are Turning to Matchmakers</t>
+          <t>The Knoxville Matchmaker for Marriage-Minded Professionals</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Boise, Explained</t>
+          <t>Serious About Dating in Boise? A Matchmaker Can Help</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker Worth It in Des Moines?</t>
+          <t>Finding Love in Des Moines With a Professional Matchmaker</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Matchmaking in Spokane for Busy Professionals</t>
+          <t>A Spokane Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -6415,7 +6415,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>What a Reno Matchmaker Actually Does</t>
+          <t>Reno Matchmaker: How Personalized Matchmaking Works</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Naples</t>
+          <t>Looking for a Matchmaker in Naples? Here's How to Choose</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">

</xml_diff>

<commit_message>
MM deck: Portland kw fix + Washington DC disambiguation
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -1809,7 +1809,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker in Washington Worth It? An Honest Take</t>
+          <t>Is Hiring a Matchmaker in DC Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Date Ideas in Washington That Actually Lead Somewhere</t>
+          <t>Date Ideas in Washington, DC That Actually Lead Somewhere</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Date Night Done Right in Washington: Ideas That Land</t>
+          <t>Date Night Done Right in Washington, DC: Ideas That Land</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>A Smarter Approach to Dating in Washington for Professionals</t>
+          <t>A Smarter Approach to Dating in DC for Professionals</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -4999,18 +4999,18 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>cara matchmaking portland me</t>
+          <t>portland matchmaker</t>
         </is>
       </c>
       <c r="D91" s="4" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F91" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>15</v>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="K91" s="7" t="inlineStr">
         <is>
-          <t>Portland (2.5M metro) — links up to the Portland location page.</t>
+          <t>Portland (2.5M metro) — clean 'portland matchmaker' (Portland OR); replaced bad kw 'cara matchmaking portland me' (Portland ME + competitor brand).</t>
         </is>
       </c>
     </row>
@@ -22377,18 +22377,18 @@
     <row r="481">
       <c r="A481" s="3" t="inlineStr">
         <is>
-          <t>cara matchmaking portland me</t>
+          <t>portland matchmaker</t>
         </is>
       </c>
       <c r="B481" s="4" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="C481" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D481" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>15</v>
+      </c>
+      <c r="D481" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="E481" s="6" t="inlineStr">
@@ -23930,7 +23930,7 @@
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  120 articles, split exactly 40/40/40 across Months 1-3
-  36,700 total monthly searches addressed
+  36,910 total monthly searches addressed
   114 easy wins at KD &lt; 30 — front-loaded into Month 1 so you see local rankings early
   Average difficulty KD 16.0 — deliberately achievable, weighted toward winnable local terms</t>
         </is>

</xml_diff>

<commit_message>
MM deck: keyword-forward single-page city titles
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Finding Love in Detroit With a Professional Matchmaker</t>
+          <t>How to Find a Matchmaker in Detroit You Can Actually Trust</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Serious About Dating in Sacramento? A Matchmaker Can Help</t>
+          <t>The Sacramento Matchmaker for Marriage-Minded Professionals</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Finding Love in Pittsburgh With a Professional Matchmaker</t>
+          <t>Meet Someone Worth Your Time With a Pittsburgh Matchmaker</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Why Cleveland Singles Are Choosing Professional Matchmakers</t>
+          <t>What a Cleveland Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Serious About Dating in Memphis? A Matchmaker Can Help</t>
+          <t>A Memphis Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Finding Love in Richmond With a Professional Matchmaker</t>
+          <t>Is a Richmond Matchmaker Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Serious About Dating in Boise? A Matchmaker Can Help</t>
+          <t>Is a Boise Matchmaker Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Finding Love in Des Moines With a Professional Matchmaker</t>
+          <t>How to Find a Matchmaker in Des Moines You Can Actually Trust</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">

</xml_diff>

<commit_message>
MM deck: affluent-enclave swap (16 cities)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -5190,12 +5190,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Cincinnati Matchmaker: How Personalized Matchmaking Works</t>
+          <t>Looking for a Matchmaker in Kansas City? Here's How to Choose</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>cincinnati matchmaker</t>
+          <t>kansas city matchmaker</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="K95" s="7" t="inlineStr">
         <is>
-          <t>Cincinnati (2.3M metro) — links up to the Cincinnati location page.</t>
+          <t>Kansas City (2.2M metro) — links up to the Kansas City location page.</t>
         </is>
       </c>
     </row>
@@ -5239,19 +5239,19 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Kansas City? Here's How to Choose</t>
+          <t>How to Find a Matchmaker in Columbus You Can Actually Trust</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>kansas city matchmaker</t>
+          <t>matchmaker columbus ohio</t>
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="K96" s="7" t="inlineStr">
         <is>
-          <t>Kansas City (2.2M metro) — links up to the Kansas City location page.</t>
+          <t>Columbus (2.1M metro) — links up to the Columbus location page.</t>
         </is>
       </c>
     </row>
@@ -5288,19 +5288,19 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>How to Find a Matchmaker in Columbus You Can Actually Trust</t>
+          <t>Professional Matchmaking in Indianapolis: What to Expect</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>matchmaker columbus ohio</t>
+          <t>indianapolis matchmaker</t>
         </is>
       </c>
       <c r="D97" s="4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="K97" s="7" t="inlineStr">
         <is>
-          <t>Columbus (2.1M metro) — links up to the Columbus location page.</t>
+          <t>Indianapolis (2.1M metro) — links up to the Indianapolis location page.</t>
         </is>
       </c>
     </row>
@@ -5337,12 +5337,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>What a Cleveland Matchmaker Does That Dating Apps Can't</t>
+          <t>Is Hiring a Matchmaker in Nashville Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>cleveland matchmaker</t>
+          <t>nashville matchmaker</t>
         </is>
       </c>
       <c r="D98" s="4" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="K98" s="7" t="inlineStr">
         <is>
-          <t>Cleveland (2.1M metro) — links up to the Cleveland location page.</t>
+          <t>Nashville (2.0M metro) — links up to the Nashville location page.</t>
         </is>
       </c>
     </row>
@@ -5386,12 +5386,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Indianapolis: What to Expect</t>
+          <t>What a Jacksonville Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>indianapolis matchmaker</t>
+          <t>jacksonville matchmaker</t>
         </is>
       </c>
       <c r="D99" s="4" t="n">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="K99" s="7" t="inlineStr">
         <is>
-          <t>Indianapolis (2.1M metro) — links up to the Indianapolis location page.</t>
+          <t>Jacksonville (1.6M metro) — links up to the Jacksonville location page.</t>
         </is>
       </c>
     </row>
@@ -5435,12 +5435,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker in Nashville Worth It? An Honest Take</t>
+          <t>Meet Someone Worth Your Time With an Oklahoma City Matchmaker</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>nashville matchmaker</t>
+          <t>oklahoma city matchmaker</t>
         </is>
       </c>
       <c r="D100" s="4" t="n">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="K100" s="7" t="inlineStr">
         <is>
-          <t>Nashville (2.0M metro) — links up to the Nashville location page.</t>
+          <t>Oklahoma City (1.4M metro) — links up to the Oklahoma City location page.</t>
         </is>
       </c>
     </row>
@@ -5484,19 +5484,19 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Matchmaking in Milwaukee for Busy, Relationship-Ready Singles</t>
+          <t>A Memphis Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>milwaukee matchmaker</t>
+          <t>matchmaker memphis</t>
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="K101" s="7" t="inlineStr">
         <is>
-          <t>Milwaukee (1.6M metro) — links up to the Milwaukee location page.</t>
+          <t>Memphis (1.3M metro) — links up to the Memphis location page.</t>
         </is>
       </c>
     </row>
@@ -5533,12 +5533,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>What a Jacksonville Matchmaker Does That Dating Apps Can't</t>
+          <t>Is a Richmond Matchmaker Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>jacksonville matchmaker</t>
+          <t>richmond matchmaker</t>
         </is>
       </c>
       <c r="D102" s="4" t="n">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="K102" s="7" t="inlineStr">
         <is>
-          <t>Jacksonville (1.6M metro) — links up to the Jacksonville location page.</t>
+          <t>Richmond (1.3M metro) — links up to the Richmond location page.</t>
         </is>
       </c>
     </row>
@@ -5582,19 +5582,19 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Meet Someone Worth Your Time With an Oklahoma City Matchmaker</t>
+          <t>A New Orleans Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>oklahoma city matchmaker</t>
+          <t>new orleans matchmaker</t>
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="K103" s="7" t="inlineStr">
         <is>
-          <t>Oklahoma City (1.4M metro) — links up to the Oklahoma City location page.</t>
+          <t>New Orleans (1.3M metro) — links up to the New Orleans location page.</t>
         </is>
       </c>
     </row>
@@ -5631,19 +5631,19 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>The Raleigh Matchmaker for Marriage-Minded Professionals</t>
+          <t>Professional Matchmaking in Salt Lake City: What to Expect</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>raleigh matchmaker</t>
+          <t>matchmaker salt lake city</t>
         </is>
       </c>
       <c r="D104" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="K104" s="7" t="inlineStr">
         <is>
-          <t>Raleigh (1.4M metro) — links up to the Raleigh location page.</t>
+          <t>Salt Lake City (1.2M metro) — links up to the Salt Lake City location page.</t>
         </is>
       </c>
     </row>
@@ -5680,19 +5680,19 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>A Memphis Matchmaker's Approach to Intentional Dating</t>
+          <t>Looking for a Matchmaker in Naples? Here's How to Choose</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>matchmaker memphis</t>
+          <t>naples matchmaker</t>
         </is>
       </c>
       <c r="D105" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="K105" s="7" t="inlineStr">
         <is>
-          <t>Memphis (1.3M metro) — links up to the Memphis location page.</t>
+          <t>Naples (0.38M metro) — links up to the Naples location page.</t>
         </is>
       </c>
     </row>
@@ -5729,19 +5729,19 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Is a Richmond Matchmaker Worth It? An Honest Take</t>
+          <t>Beverly Hills Matchmaker: Discreet, High-End Introductions</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>richmond matchmaker</t>
+          <t>beverly hills matchmaker</t>
         </is>
       </c>
       <c r="D106" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
       </c>
       <c r="K106" s="7" t="inlineStr">
         <is>
-          <t>Richmond (1.3M metro) — links up to the Richmond location page.</t>
+          <t>Beverly Hills (affluent enclave) — links up to the Los Angeles metro.</t>
         </is>
       </c>
     </row>
@@ -5778,19 +5778,19 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>A New Orleans Matchmaker's Approach to Intentional Dating</t>
+          <t>Looking for a Matchmaker in Malibu?</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>new orleans matchmaker</t>
+          <t>malibu matchmaker</t>
         </is>
       </c>
       <c r="D107" s="4" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
@@ -5817,7 +5817,7 @@
       </c>
       <c r="K107" s="7" t="inlineStr">
         <is>
-          <t>New Orleans (1.3M metro) — links up to the New Orleans location page.</t>
+          <t>Malibu (affluent enclave) — links up to the Los Angeles metro.</t>
         </is>
       </c>
     </row>
@@ -5827,12 +5827,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Louisville Matchmaker: How Personalized Matchmaking Works</t>
+          <t>Your Personal Matchmaker in Newport Beach</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>louisville matchmaker</t>
+          <t>newport beach matchmaker</t>
         </is>
       </c>
       <c r="D108" s="4" t="n">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="K108" s="7" t="inlineStr">
         <is>
-          <t>Louisville (1.3M metro) — links up to the Louisville location page.</t>
+          <t>Newport Beach (affluent enclave) — links up to the Los Angeles metro / California state.</t>
         </is>
       </c>
     </row>
@@ -5876,19 +5876,19 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Buffalo? Here's How to Choose</t>
+          <t>San Jose Matchmaking for Discerning Singles</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>buffalo matchmaker</t>
+          <t>matchmaker san jose</t>
         </is>
       </c>
       <c r="D109" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="K109" s="7" t="inlineStr">
         <is>
-          <t>Buffalo (1.2M metro) — links up to the Buffalo location page.</t>
+          <t>San Jose (affluent enclave) — links up to the San Francisco / Bay Area metro.</t>
         </is>
       </c>
     </row>
@@ -5925,19 +5925,19 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Salt Lake City: What to Expect</t>
+          <t>How to Find a Matchmaker in Palo Alto You Can Trust</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>matchmaker salt lake city</t>
+          <t>palo alto matchmaker</t>
         </is>
       </c>
       <c r="D110" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="K110" s="7" t="inlineStr">
         <is>
-          <t>Salt Lake City (1.2M metro) — links up to the Salt Lake City location page.</t>
+          <t>Palo Alto (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -5974,12 +5974,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker in Birmingham Worth It? An Honest Take</t>
+          <t>The Atherton Matchmaker for Marriage-Minded Singles</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>birmingham matchmaker</t>
+          <t>atherton matchmaker</t>
         </is>
       </c>
       <c r="D111" s="4" t="n">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="K111" s="7" t="inlineStr">
         <is>
-          <t>Birmingham (1.1M metro) — links up to the Birmingham location page.</t>
+          <t>Atherton (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -6023,19 +6023,19 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Matchmaking in Tucson for Busy, Relationship-Ready Singles</t>
+          <t>Meet Your Match With a Hillsborough Matchmaker</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>matchmaker tucson</t>
+          <t>hillsborough matchmaker</t>
         </is>
       </c>
       <c r="D112" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="K112" s="7" t="inlineStr">
         <is>
-          <t>Tucson (1.05M metro) — links up to the Tucson location page.</t>
+          <t>Hillsborough (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -6072,19 +6072,19 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>What a Tulsa Matchmaker Does That Dating Apps Can't</t>
+          <t>Elite Matchmaking in Los Altos, Done for You</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>tulsa matchmaker</t>
+          <t>los altos matchmaker</t>
         </is>
       </c>
       <c r="D113" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="K113" s="7" t="inlineStr">
         <is>
-          <t>Tulsa (1.02M metro) — links up to the Tulsa location page.</t>
+          <t>Los Altos (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -6121,19 +6121,19 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Omaha: Introductions Done Right</t>
+          <t>Scarsdale Matchmaker: Discreet, High-End Introductions</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>omaha matchmaker</t>
+          <t>scarsdale matchmaker</t>
         </is>
       </c>
       <c r="D114" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="K114" s="7" t="inlineStr">
         <is>
-          <t>Omaha (0.97M metro) — links up to the Omaha location page.</t>
+          <t>Scarsdale (affluent enclave) — links up to the New York metro.</t>
         </is>
       </c>
     </row>
@@ -6170,19 +6170,19 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Meet Someone Worth Your Time With an Albuquerque Matchmaker</t>
+          <t>Looking for a Matchmaker in the Hamptons?</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>matchmaker albuquerque</t>
+          <t>hamptons matchmaker</t>
         </is>
       </c>
       <c r="D115" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
       </c>
       <c r="K115" s="7" t="inlineStr">
         <is>
-          <t>Albuquerque (0.92M metro) — links up to the Albuquerque location page.</t>
+          <t>Hamptons (affluent enclave) — links up to the New York metro.</t>
         </is>
       </c>
     </row>
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>The Knoxville Matchmaker for Marriage-Minded Professionals</t>
+          <t>Your Personal Matchmaker in Greenwich</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>knoxville matchmaker</t>
+          <t>greenwich matchmaker</t>
         </is>
       </c>
       <c r="D116" s="4" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="K116" s="7" t="inlineStr">
         <is>
-          <t>Knoxville (0.87M metro) — links up to the Knoxville location page.</t>
+          <t>Greenwich (affluent enclave) — links up to the New York metro / Connecticut state.</t>
         </is>
       </c>
     </row>
@@ -6268,12 +6268,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Is a Boise Matchmaker Worth It? An Honest Take</t>
+          <t>Darien Matchmaking for Discerning Singles</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>boise matchmaker</t>
+          <t>darien matchmaker</t>
         </is>
       </c>
       <c r="D117" s="4" t="n">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="K117" s="7" t="inlineStr">
         <is>
-          <t>Boise (0.76M metro) — links up to the Boise location page.</t>
+          <t>Darien (affluent enclave) — links up to the New York metro / Connecticut state.</t>
         </is>
       </c>
     </row>
@@ -6317,12 +6317,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>How to Find a Matchmaker in Des Moines You Can Actually Trust</t>
+          <t>How to Find a Matchmaker in Short Hills You Can Trust</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>des moines matchmaker</t>
+          <t>short hills matchmaker</t>
         </is>
       </c>
       <c r="D118" s="4" t="n">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="K118" s="7" t="inlineStr">
         <is>
-          <t>Des Moines (0.71M metro) — links up to the Des Moines location page.</t>
+          <t>Short Hills (affluent enclave) — links up to the New York metro / New Jersey state.</t>
         </is>
       </c>
     </row>
@@ -6366,12 +6366,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>A Spokane Matchmaker's Approach to Intentional Dating</t>
+          <t>The McLean Matchmaker for Marriage-Minded Singles</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>spokane matchmaker</t>
+          <t>mclean matchmaker</t>
         </is>
       </c>
       <c r="D119" s="4" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="K119" s="7" t="inlineStr">
         <is>
-          <t>Spokane (0.6M metro) — links up to the Spokane location page.</t>
+          <t>McLean (affluent enclave) — links up to the Washington DC metro / Virginia state.</t>
         </is>
       </c>
     </row>
@@ -6415,12 +6415,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Reno Matchmaker: How Personalized Matchmaking Works</t>
+          <t>Meet Your Match With a Boca Raton Matchmaker</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>reno matchmaker</t>
+          <t>boca raton matchmaker</t>
         </is>
       </c>
       <c r="D120" s="4" t="n">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="K120" s="7" t="inlineStr">
         <is>
-          <t>Reno (0.49M metro) — links up to the Reno location page.</t>
+          <t>Boca Raton (affluent enclave) — links up to the Miami metro / Florida state.</t>
         </is>
       </c>
     </row>
@@ -6464,12 +6464,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Naples? Here's How to Choose</t>
+          <t>Elite Matchmaking in Park City, Done for You</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>naples matchmaker</t>
+          <t>park city matchmaker</t>
         </is>
       </c>
       <c r="D121" s="4" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K121" s="7" t="inlineStr">
         <is>
-          <t>Naples (0.38M metro) — links up to the Naples location page.</t>
+          <t>Park City (affluent enclave) — links up to the Salt Lake City metro / Utah state.</t>
         </is>
       </c>
     </row>
@@ -22509,7 +22509,7 @@
     <row r="485">
       <c r="A485" s="3" t="inlineStr">
         <is>
-          <t>cincinnati matchmaker</t>
+          <t>kansas city matchmaker</t>
         </is>
       </c>
       <c r="B485" s="4" t="n">
@@ -22542,14 +22542,14 @@
     <row r="486">
       <c r="A486" s="3" t="inlineStr">
         <is>
-          <t>kansas city matchmaker</t>
+          <t>matchmaker columbus ohio</t>
         </is>
       </c>
       <c r="B486" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="C486" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D486" s="10" t="inlineStr">
         <is>
@@ -22575,14 +22575,14 @@
     <row r="487">
       <c r="A487" s="3" t="inlineStr">
         <is>
-          <t>matchmaker columbus ohio</t>
+          <t>indianapolis matchmaker</t>
         </is>
       </c>
       <c r="B487" s="4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C487" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D487" s="10" t="inlineStr">
         <is>
@@ -22608,7 +22608,7 @@
     <row r="488">
       <c r="A488" s="3" t="inlineStr">
         <is>
-          <t>cleveland matchmaker</t>
+          <t>nashville matchmaker</t>
         </is>
       </c>
       <c r="B488" s="4" t="n">
@@ -22641,7 +22641,7 @@
     <row r="489">
       <c r="A489" s="3" t="inlineStr">
         <is>
-          <t>indianapolis matchmaker</t>
+          <t>jacksonville matchmaker</t>
         </is>
       </c>
       <c r="B489" s="4" t="n">
@@ -22674,7 +22674,7 @@
     <row r="490">
       <c r="A490" s="3" t="inlineStr">
         <is>
-          <t>nashville matchmaker</t>
+          <t>oklahoma city matchmaker</t>
         </is>
       </c>
       <c r="B490" s="4" t="n">
@@ -22707,14 +22707,14 @@
     <row r="491">
       <c r="A491" s="3" t="inlineStr">
         <is>
-          <t>milwaukee matchmaker</t>
+          <t>matchmaker memphis</t>
         </is>
       </c>
       <c r="B491" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C491" s="2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D491" s="10" t="inlineStr">
         <is>
@@ -22740,7 +22740,7 @@
     <row r="492">
       <c r="A492" s="3" t="inlineStr">
         <is>
-          <t>jacksonville matchmaker</t>
+          <t>richmond matchmaker</t>
         </is>
       </c>
       <c r="B492" s="4" t="n">
@@ -22773,14 +22773,14 @@
     <row r="493">
       <c r="A493" s="3" t="inlineStr">
         <is>
-          <t>oklahoma city matchmaker</t>
+          <t>new orleans matchmaker</t>
         </is>
       </c>
       <c r="B493" s="4" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="C493" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D493" s="10" t="inlineStr">
         <is>
@@ -22806,14 +22806,14 @@
     <row r="494">
       <c r="A494" s="3" t="inlineStr">
         <is>
-          <t>raleigh matchmaker</t>
+          <t>matchmaker salt lake city</t>
         </is>
       </c>
       <c r="B494" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C494" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D494" s="10" t="inlineStr">
         <is>
@@ -22839,14 +22839,14 @@
     <row r="495">
       <c r="A495" s="3" t="inlineStr">
         <is>
-          <t>matchmaker memphis</t>
+          <t>naples matchmaker</t>
         </is>
       </c>
       <c r="B495" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C495" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D495" s="10" t="inlineStr">
         <is>
@@ -22872,14 +22872,14 @@
     <row r="496">
       <c r="A496" s="3" t="inlineStr">
         <is>
-          <t>richmond matchmaker</t>
+          <t>beverly hills matchmaker</t>
         </is>
       </c>
       <c r="B496" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C496" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D496" s="10" t="inlineStr">
         <is>
@@ -22905,14 +22905,14 @@
     <row r="497">
       <c r="A497" s="3" t="inlineStr">
         <is>
-          <t>new orleans matchmaker</t>
+          <t>malibu matchmaker</t>
         </is>
       </c>
       <c r="B497" s="4" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C497" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D497" s="10" t="inlineStr">
         <is>
@@ -22938,7 +22938,7 @@
     <row r="498">
       <c r="A498" s="3" t="inlineStr">
         <is>
-          <t>louisville matchmaker</t>
+          <t>newport beach matchmaker</t>
         </is>
       </c>
       <c r="B498" s="4" t="n">
@@ -22971,14 +22971,14 @@
     <row r="499">
       <c r="A499" s="3" t="inlineStr">
         <is>
-          <t>buffalo matchmaker</t>
+          <t>matchmaker san jose</t>
         </is>
       </c>
       <c r="B499" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C499" s="2" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D499" s="10" t="inlineStr">
         <is>
@@ -23004,14 +23004,14 @@
     <row r="500">
       <c r="A500" s="3" t="inlineStr">
         <is>
-          <t>matchmaker salt lake city</t>
+          <t>palo alto matchmaker</t>
         </is>
       </c>
       <c r="B500" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C500" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D500" s="10" t="inlineStr">
         <is>
@@ -23037,7 +23037,7 @@
     <row r="501">
       <c r="A501" s="3" t="inlineStr">
         <is>
-          <t>birmingham matchmaker</t>
+          <t>atherton matchmaker</t>
         </is>
       </c>
       <c r="B501" s="4" t="n">
@@ -23070,14 +23070,14 @@
     <row r="502">
       <c r="A502" s="3" t="inlineStr">
         <is>
-          <t>matchmaker tucson</t>
+          <t>hillsborough matchmaker</t>
         </is>
       </c>
       <c r="B502" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C502" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D502" s="10" t="inlineStr">
         <is>
@@ -23103,14 +23103,14 @@
     <row r="503">
       <c r="A503" s="3" t="inlineStr">
         <is>
-          <t>tulsa matchmaker</t>
+          <t>los altos matchmaker</t>
         </is>
       </c>
       <c r="B503" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C503" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D503" s="10" t="inlineStr">
         <is>
@@ -23136,14 +23136,14 @@
     <row r="504">
       <c r="A504" s="3" t="inlineStr">
         <is>
-          <t>omaha matchmaker</t>
+          <t>scarsdale matchmaker</t>
         </is>
       </c>
       <c r="B504" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C504" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D504" s="10" t="inlineStr">
         <is>
@@ -23169,14 +23169,14 @@
     <row r="505">
       <c r="A505" s="3" t="inlineStr">
         <is>
-          <t>matchmaker albuquerque</t>
+          <t>hamptons matchmaker</t>
         </is>
       </c>
       <c r="B505" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C505" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D505" s="10" t="inlineStr">
         <is>
@@ -23202,7 +23202,7 @@
     <row r="506">
       <c r="A506" s="3" t="inlineStr">
         <is>
-          <t>knoxville matchmaker</t>
+          <t>greenwich matchmaker</t>
         </is>
       </c>
       <c r="B506" s="4" t="n">
@@ -23235,7 +23235,7 @@
     <row r="507">
       <c r="A507" s="3" t="inlineStr">
         <is>
-          <t>boise matchmaker</t>
+          <t>darien matchmaker</t>
         </is>
       </c>
       <c r="B507" s="4" t="n">
@@ -23268,7 +23268,7 @@
     <row r="508">
       <c r="A508" s="3" t="inlineStr">
         <is>
-          <t>des moines matchmaker</t>
+          <t>short hills matchmaker</t>
         </is>
       </c>
       <c r="B508" s="4" t="n">
@@ -23301,7 +23301,7 @@
     <row r="509">
       <c r="A509" s="3" t="inlineStr">
         <is>
-          <t>spokane matchmaker</t>
+          <t>mclean matchmaker</t>
         </is>
       </c>
       <c r="B509" s="4" t="n">
@@ -23334,7 +23334,7 @@
     <row r="510">
       <c r="A510" s="3" t="inlineStr">
         <is>
-          <t>reno matchmaker</t>
+          <t>boca raton matchmaker</t>
         </is>
       </c>
       <c r="B510" s="4" t="n">
@@ -23367,7 +23367,7 @@
     <row r="511">
       <c r="A511" s="3" t="inlineStr">
         <is>
-          <t>naples matchmaker</t>
+          <t>park city matchmaker</t>
         </is>
       </c>
       <c r="B511" s="4" t="n">
@@ -23830,7 +23830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="114" customWidth="1" min="1" max="1"/>
@@ -23930,7 +23930,7 @@
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  120 articles, split exactly 40/40/40 across Months 1-3
-  36,910 total monthly searches addressed
+  36,870 total monthly searches addressed
   114 easy wins at KD &lt; 30 — front-loaded into Month 1 so you see local rankings early
   Average difficulty KD 16.0 — deliberately achievable, weighted toward winnable local terms</t>
         </is>
@@ -23939,12 +23939,31 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
+          <t>Why some cities show low or zero search volume (and why that's fine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="98" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>You'll notice the smaller metros show low or even zero measurable monthly searches. That's expected — matchmaking is a
+niche, so most cities only have real search demand for one term: '[city] matchmaker.' These pages aren't a traffic play;
+they're a local-presence and AI-citation play — being the name that comes up when someone asks Google's AI or ChatGPT
+'who's a matchmaker in [city]?', and holding the local map spot. Depth follows demand: the biggest metros get a full
+cluster of pages, the smallest get one focused, fully-optimized page. Every city you serve is covered — we simply size
+each city's content to its actual demand so the budget goes where the return is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="56" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+    <row r="23" ht="56" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>See the 'Excluded' sheet. The big buckets: generic non-local listicle terms ('date night ideas', 450K vol, zero buyer
 intent), dating-app and free-tool searches (your buyer has left apps behind), TV-show entertainment searches
@@ -23952,15 +23971,15 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="56" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="26" ht="56" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Approve the 120-article plan and ClusterMagic begins the Month 1 batch within 5 business days. Articles are
 entity-rich, internally linked, schema-marked, and shipped to your CMS as drafts for review — built to win both

</xml_diff>

<commit_message>
MM deck: affluent-suburb swap (Highland Park/Southlake/Great Falls/Hinsdale)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -5043,23 +5043,23 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>The Sacramento Matchmaker for Marriage-Minded Professionals</t>
+          <t>Meet Someone Worth Your Time With a Pittsburgh Matchmaker</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>sacramento matchmaker</t>
+          <t>pittsburgh matchmaker</t>
         </is>
       </c>
       <c r="D92" s="4" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F92" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>29</v>
+      </c>
+      <c r="F92" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G92" s="6" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="K92" s="7" t="inlineStr">
         <is>
-          <t>Sacramento (2.4M metro) — links up to the Sacramento location page.</t>
+          <t>Pittsburgh (2.3M metro) — links up to the Pittsburgh location page.</t>
         </is>
       </c>
     </row>
@@ -5092,23 +5092,23 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Meet Someone Worth Your Time With a Pittsburgh Matchmaker</t>
+          <t>A Las Vegas Matchmaker's Approach to Intentional Dating</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>pittsburgh matchmaker</t>
+          <t>las vegas matchmaker</t>
         </is>
       </c>
       <c r="D93" s="4" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="F93" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>15</v>
+      </c>
+      <c r="F93" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="K93" s="7" t="inlineStr">
         <is>
-          <t>Pittsburgh (2.3M metro) — links up to the Pittsburgh location page.</t>
+          <t>Las Vegas (2.3M metro) — links up to the Las Vegas location page.</t>
         </is>
       </c>
     </row>
@@ -5141,12 +5141,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>A Las Vegas Matchmaker's Approach to Intentional Dating</t>
+          <t>Looking for a Matchmaker in Kansas City? Here's How to Choose</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>las vegas matchmaker</t>
+          <t>kansas city matchmaker</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="K94" s="7" t="inlineStr">
         <is>
-          <t>Las Vegas (2.3M metro) — links up to the Las Vegas location page.</t>
+          <t>Kansas City (2.2M metro) — links up to the Kansas City location page.</t>
         </is>
       </c>
     </row>
@@ -5190,19 +5190,19 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Kansas City? Here's How to Choose</t>
+          <t>How to Find a Matchmaker in Columbus You Can Actually Trust</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>kansas city matchmaker</t>
+          <t>matchmaker columbus ohio</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="K95" s="7" t="inlineStr">
         <is>
-          <t>Kansas City (2.2M metro) — links up to the Kansas City location page.</t>
+          <t>Columbus (2.1M metro) — links up to the Columbus location page.</t>
         </is>
       </c>
     </row>
@@ -5239,19 +5239,19 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>How to Find a Matchmaker in Columbus You Can Actually Trust</t>
+          <t>Professional Matchmaking in Indianapolis: What to Expect</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>matchmaker columbus ohio</t>
+          <t>indianapolis matchmaker</t>
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="K96" s="7" t="inlineStr">
         <is>
-          <t>Columbus (2.1M metro) — links up to the Columbus location page.</t>
+          <t>Indianapolis (2.1M metro) — links up to the Indianapolis location page.</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Indianapolis: What to Expect</t>
+          <t>Is Hiring a Matchmaker in Nashville Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>indianapolis matchmaker</t>
+          <t>nashville matchmaker</t>
         </is>
       </c>
       <c r="D97" s="4" t="n">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="K97" s="7" t="inlineStr">
         <is>
-          <t>Indianapolis (2.1M metro) — links up to the Indianapolis location page.</t>
+          <t>Nashville (2.0M metro) — links up to the Nashville location page.</t>
         </is>
       </c>
     </row>
@@ -5337,12 +5337,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Is Hiring a Matchmaker in Nashville Worth It? An Honest Take</t>
+          <t>What a Jacksonville Matchmaker Does That Dating Apps Can't</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>nashville matchmaker</t>
+          <t>jacksonville matchmaker</t>
         </is>
       </c>
       <c r="D98" s="4" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="K98" s="7" t="inlineStr">
         <is>
-          <t>Nashville (2.0M metro) — links up to the Nashville location page.</t>
+          <t>Jacksonville (1.6M metro) — links up to the Jacksonville location page.</t>
         </is>
       </c>
     </row>
@@ -5386,12 +5386,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>What a Jacksonville Matchmaker Does That Dating Apps Can't</t>
+          <t>Is a Richmond Matchmaker Worth It? An Honest Take</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>jacksonville matchmaker</t>
+          <t>richmond matchmaker</t>
         </is>
       </c>
       <c r="D99" s="4" t="n">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="K99" s="7" t="inlineStr">
         <is>
-          <t>Jacksonville (1.6M metro) — links up to the Jacksonville location page.</t>
+          <t>Richmond (1.3M metro) — links up to the Richmond location page.</t>
         </is>
       </c>
     </row>
@@ -5435,19 +5435,19 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Meet Someone Worth Your Time With an Oklahoma City Matchmaker</t>
+          <t>Professional Matchmaking in Salt Lake City: What to Expect</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>oklahoma city matchmaker</t>
+          <t>matchmaker salt lake city</t>
         </is>
       </c>
       <c r="D100" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
@@ -5474,7 +5474,7 @@
       </c>
       <c r="K100" s="7" t="inlineStr">
         <is>
-          <t>Oklahoma City (1.4M metro) — links up to the Oklahoma City location page.</t>
+          <t>Salt Lake City (1.2M metro) — links up to the Salt Lake City location page.</t>
         </is>
       </c>
     </row>
@@ -5484,19 +5484,19 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>A Memphis Matchmaker's Approach to Intentional Dating</t>
+          <t>Looking for a Matchmaker in Naples? Here's How to Choose</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>matchmaker memphis</t>
+          <t>naples matchmaker</t>
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="K101" s="7" t="inlineStr">
         <is>
-          <t>Memphis (1.3M metro) — links up to the Memphis location page.</t>
+          <t>Naples (0.38M metro) — links up to the Naples location page.</t>
         </is>
       </c>
     </row>
@@ -5533,19 +5533,19 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Is a Richmond Matchmaker Worth It? An Honest Take</t>
+          <t>Beverly Hills Matchmaker: Discreet, High-End Introductions</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>richmond matchmaker</t>
+          <t>beverly hills matchmaker</t>
         </is>
       </c>
       <c r="D102" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="K102" s="7" t="inlineStr">
         <is>
-          <t>Richmond (1.3M metro) — links up to the Richmond location page.</t>
+          <t>Beverly Hills (affluent enclave) — links up to the Los Angeles metro.</t>
         </is>
       </c>
     </row>
@@ -5582,19 +5582,19 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>A New Orleans Matchmaker's Approach to Intentional Dating</t>
+          <t>Looking for a Matchmaker in Malibu?</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>new orleans matchmaker</t>
+          <t>malibu matchmaker</t>
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="K103" s="7" t="inlineStr">
         <is>
-          <t>New Orleans (1.3M metro) — links up to the New Orleans location page.</t>
+          <t>Malibu (affluent enclave) — links up to the Los Angeles metro.</t>
         </is>
       </c>
     </row>
@@ -5631,19 +5631,19 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Professional Matchmaking in Salt Lake City: What to Expect</t>
+          <t>Your Personal Matchmaker in Newport Beach</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>matchmaker salt lake city</t>
+          <t>newport beach matchmaker</t>
         </is>
       </c>
       <c r="D104" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="K104" s="7" t="inlineStr">
         <is>
-          <t>Salt Lake City (1.2M metro) — links up to the Salt Lake City location page.</t>
+          <t>Newport Beach (affluent enclave) — links up to the Los Angeles metro / California state.</t>
         </is>
       </c>
     </row>
@@ -5680,19 +5680,19 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Naples? Here's How to Choose</t>
+          <t>San Jose Matchmaking for Discerning Singles</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>naples matchmaker</t>
+          <t>matchmaker san jose</t>
         </is>
       </c>
       <c r="D105" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="K105" s="7" t="inlineStr">
         <is>
-          <t>Naples (0.38M metro) — links up to the Naples location page.</t>
+          <t>San Jose (affluent enclave) — links up to the San Francisco / Bay Area metro.</t>
         </is>
       </c>
     </row>
@@ -5729,19 +5729,19 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Beverly Hills Matchmaker: Discreet, High-End Introductions</t>
+          <t>How to Find a Matchmaker in Palo Alto You Can Trust</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>beverly hills matchmaker</t>
+          <t>palo alto matchmaker</t>
         </is>
       </c>
       <c r="D106" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
       </c>
       <c r="K106" s="7" t="inlineStr">
         <is>
-          <t>Beverly Hills (affluent enclave) — links up to the Los Angeles metro.</t>
+          <t>Palo Alto (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -5778,12 +5778,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in Malibu?</t>
+          <t>The Atherton Matchmaker for Marriage-Minded Singles</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>malibu matchmaker</t>
+          <t>atherton matchmaker</t>
         </is>
       </c>
       <c r="D107" s="4" t="n">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="K107" s="7" t="inlineStr">
         <is>
-          <t>Malibu (affluent enclave) — links up to the Los Angeles metro.</t>
+          <t>Atherton (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -5827,12 +5827,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Newport Beach</t>
+          <t>Meet Your Match With a Hillsborough Matchmaker</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>newport beach matchmaker</t>
+          <t>hillsborough matchmaker</t>
         </is>
       </c>
       <c r="D108" s="4" t="n">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="K108" s="7" t="inlineStr">
         <is>
-          <t>Newport Beach (affluent enclave) — links up to the Los Angeles metro / California state.</t>
+          <t>Hillsborough (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -5876,19 +5876,19 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>San Jose Matchmaking for Discerning Singles</t>
+          <t>Elite Matchmaking in Los Altos, Done for You</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>matchmaker san jose</t>
+          <t>los altos matchmaker</t>
         </is>
       </c>
       <c r="D109" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="K109" s="7" t="inlineStr">
         <is>
-          <t>San Jose (affluent enclave) — links up to the San Francisco / Bay Area metro.</t>
+          <t>Los Altos (affluent enclave) — links up to the San Francisco metro.</t>
         </is>
       </c>
     </row>
@@ -5925,12 +5925,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>How to Find a Matchmaker in Palo Alto You Can Trust</t>
+          <t>Scarsdale Matchmaker: Discreet, High-End Introductions</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>palo alto matchmaker</t>
+          <t>scarsdale matchmaker</t>
         </is>
       </c>
       <c r="D110" s="4" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="K110" s="7" t="inlineStr">
         <is>
-          <t>Palo Alto (affluent enclave) — links up to the San Francisco metro.</t>
+          <t>Scarsdale (affluent enclave) — links up to the New York metro.</t>
         </is>
       </c>
     </row>
@@ -5974,12 +5974,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>The Atherton Matchmaker for Marriage-Minded Singles</t>
+          <t>Looking for a Matchmaker in the Hamptons?</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>atherton matchmaker</t>
+          <t>hamptons matchmaker</t>
         </is>
       </c>
       <c r="D111" s="4" t="n">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="K111" s="7" t="inlineStr">
         <is>
-          <t>Atherton (affluent enclave) — links up to the San Francisco metro.</t>
+          <t>Hamptons (affluent enclave) — links up to the New York metro.</t>
         </is>
       </c>
     </row>
@@ -6023,12 +6023,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Meet Your Match With a Hillsborough Matchmaker</t>
+          <t>Your Personal Matchmaker in Greenwich</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>hillsborough matchmaker</t>
+          <t>greenwich matchmaker</t>
         </is>
       </c>
       <c r="D112" s="4" t="n">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="K112" s="7" t="inlineStr">
         <is>
-          <t>Hillsborough (affluent enclave) — links up to the San Francisco metro.</t>
+          <t>Greenwich (affluent enclave) — links up to the New York metro / Connecticut state.</t>
         </is>
       </c>
     </row>
@@ -6072,12 +6072,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Elite Matchmaking in Los Altos, Done for You</t>
+          <t>Darien Matchmaking for Discerning Singles</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>los altos matchmaker</t>
+          <t>darien matchmaker</t>
         </is>
       </c>
       <c r="D113" s="4" t="n">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="K113" s="7" t="inlineStr">
         <is>
-          <t>Los Altos (affluent enclave) — links up to the San Francisco metro.</t>
+          <t>Darien (affluent enclave) — links up to the New York metro / Connecticut state.</t>
         </is>
       </c>
     </row>
@@ -6121,12 +6121,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Scarsdale Matchmaker: Discreet, High-End Introductions</t>
+          <t>How to Find a Matchmaker in Short Hills You Can Trust</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>scarsdale matchmaker</t>
+          <t>short hills matchmaker</t>
         </is>
       </c>
       <c r="D114" s="4" t="n">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="K114" s="7" t="inlineStr">
         <is>
-          <t>Scarsdale (affluent enclave) — links up to the New York metro.</t>
+          <t>Short Hills (affluent enclave) — links up to the New York metro / New Jersey state.</t>
         </is>
       </c>
     </row>
@@ -6170,12 +6170,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Looking for a Matchmaker in the Hamptons?</t>
+          <t>The McLean Matchmaker for Marriage-Minded Singles</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>hamptons matchmaker</t>
+          <t>mclean matchmaker</t>
         </is>
       </c>
       <c r="D115" s="4" t="n">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="K115" s="7" t="inlineStr">
         <is>
-          <t>Hamptons (affluent enclave) — links up to the New York metro.</t>
+          <t>McLean (affluent enclave) — links up to the Washington DC metro / Virginia state.</t>
         </is>
       </c>
     </row>
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Your Personal Matchmaker in Greenwich</t>
+          <t>Meet Your Match With a Boca Raton Matchmaker</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>greenwich matchmaker</t>
+          <t>boca raton matchmaker</t>
         </is>
       </c>
       <c r="D116" s="4" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="K116" s="7" t="inlineStr">
         <is>
-          <t>Greenwich (affluent enclave) — links up to the New York metro / Connecticut state.</t>
+          <t>Boca Raton (affluent enclave) — links up to the Miami metro / Florida state.</t>
         </is>
       </c>
     </row>
@@ -6268,12 +6268,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Darien Matchmaking for Discerning Singles</t>
+          <t>Elite Matchmaking in Park City, Done for You</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>darien matchmaker</t>
+          <t>park city matchmaker</t>
         </is>
       </c>
       <c r="D117" s="4" t="n">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="K117" s="7" t="inlineStr">
         <is>
-          <t>Darien (affluent enclave) — links up to the New York metro / Connecticut state.</t>
+          <t>Park City (affluent enclave) — links up to the Salt Lake City metro / Utah state.</t>
         </is>
       </c>
     </row>
@@ -6317,12 +6317,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>How to Find a Matchmaker in Short Hills You Can Trust</t>
+          <t>Highland Park, TX Matchmaker: Discreet, High-End Introductions</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>short hills matchmaker</t>
+          <t>highland park matchmaker</t>
         </is>
       </c>
       <c r="D118" s="4" t="n">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="K118" s="7" t="inlineStr">
         <is>
-          <t>Short Hills (affluent enclave) — links up to the New York metro / New Jersey state.</t>
+          <t>Highland Park, TX (affluent suburb) — links up to the Dallas metro.</t>
         </is>
       </c>
     </row>
@@ -6366,12 +6366,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>The McLean Matchmaker for Marriage-Minded Singles</t>
+          <t>Looking for a Matchmaker in Southlake, TX?</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>mclean matchmaker</t>
+          <t>southlake matchmaker</t>
         </is>
       </c>
       <c r="D119" s="4" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="K119" s="7" t="inlineStr">
         <is>
-          <t>McLean (affluent enclave) — links up to the Washington DC metro / Virginia state.</t>
+          <t>Southlake, TX (affluent suburb) — links up to the Dallas metro.</t>
         </is>
       </c>
     </row>
@@ -6415,12 +6415,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Meet Your Match With a Boca Raton Matchmaker</t>
+          <t>Your Personal Matchmaker in Great Falls, VA</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>boca raton matchmaker</t>
+          <t>great falls matchmaker</t>
         </is>
       </c>
       <c r="D120" s="4" t="n">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="K120" s="7" t="inlineStr">
         <is>
-          <t>Boca Raton (affluent enclave) — links up to the Miami metro / Florida state.</t>
+          <t>Great Falls, VA (affluent suburb) — links up to the Washington DC metro / Virginia state.</t>
         </is>
       </c>
     </row>
@@ -6464,12 +6464,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Elite Matchmaking in Park City, Done for You</t>
+          <t>Hinsdale, IL Matchmaking for Discerning Singles</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>park city matchmaker</t>
+          <t>hinsdale matchmaker</t>
         </is>
       </c>
       <c r="D121" s="4" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K121" s="7" t="inlineStr">
         <is>
-          <t>Park City (affluent enclave) — links up to the Salt Lake City metro / Utah state.</t>
+          <t>Hinsdale, IL (affluent suburb) — links up to the Chicago metro.</t>
         </is>
       </c>
     </row>
@@ -22410,18 +22410,18 @@
     <row r="482">
       <c r="A482" s="3" t="inlineStr">
         <is>
-          <t>sacramento matchmaker</t>
+          <t>pittsburgh matchmaker</t>
         </is>
       </c>
       <c r="B482" s="4" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C482" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D482" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>29</v>
+      </c>
+      <c r="D482" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E482" s="6" t="inlineStr">
@@ -22443,18 +22443,18 @@
     <row r="483">
       <c r="A483" s="3" t="inlineStr">
         <is>
-          <t>pittsburgh matchmaker</t>
+          <t>las vegas matchmaker</t>
         </is>
       </c>
       <c r="B483" s="4" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="C483" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="D483" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>15</v>
+      </c>
+      <c r="D483" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="E483" s="6" t="inlineStr">
@@ -22476,7 +22476,7 @@
     <row r="484">
       <c r="A484" s="3" t="inlineStr">
         <is>
-          <t>las vegas matchmaker</t>
+          <t>kansas city matchmaker</t>
         </is>
       </c>
       <c r="B484" s="4" t="n">
@@ -22509,14 +22509,14 @@
     <row r="485">
       <c r="A485" s="3" t="inlineStr">
         <is>
-          <t>kansas city matchmaker</t>
+          <t>matchmaker columbus ohio</t>
         </is>
       </c>
       <c r="B485" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="C485" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D485" s="10" t="inlineStr">
         <is>
@@ -22542,14 +22542,14 @@
     <row r="486">
       <c r="A486" s="3" t="inlineStr">
         <is>
-          <t>matchmaker columbus ohio</t>
+          <t>indianapolis matchmaker</t>
         </is>
       </c>
       <c r="B486" s="4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C486" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D486" s="10" t="inlineStr">
         <is>
@@ -22575,7 +22575,7 @@
     <row r="487">
       <c r="A487" s="3" t="inlineStr">
         <is>
-          <t>indianapolis matchmaker</t>
+          <t>nashville matchmaker</t>
         </is>
       </c>
       <c r="B487" s="4" t="n">
@@ -22608,7 +22608,7 @@
     <row r="488">
       <c r="A488" s="3" t="inlineStr">
         <is>
-          <t>nashville matchmaker</t>
+          <t>jacksonville matchmaker</t>
         </is>
       </c>
       <c r="B488" s="4" t="n">
@@ -22641,7 +22641,7 @@
     <row r="489">
       <c r="A489" s="3" t="inlineStr">
         <is>
-          <t>jacksonville matchmaker</t>
+          <t>richmond matchmaker</t>
         </is>
       </c>
       <c r="B489" s="4" t="n">
@@ -22674,14 +22674,14 @@
     <row r="490">
       <c r="A490" s="3" t="inlineStr">
         <is>
-          <t>oklahoma city matchmaker</t>
+          <t>matchmaker salt lake city</t>
         </is>
       </c>
       <c r="B490" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C490" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D490" s="10" t="inlineStr">
         <is>
@@ -22707,14 +22707,14 @@
     <row r="491">
       <c r="A491" s="3" t="inlineStr">
         <is>
-          <t>matchmaker memphis</t>
+          <t>naples matchmaker</t>
         </is>
       </c>
       <c r="B491" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C491" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D491" s="10" t="inlineStr">
         <is>
@@ -22740,14 +22740,14 @@
     <row r="492">
       <c r="A492" s="3" t="inlineStr">
         <is>
-          <t>richmond matchmaker</t>
+          <t>beverly hills matchmaker</t>
         </is>
       </c>
       <c r="B492" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C492" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D492" s="10" t="inlineStr">
         <is>
@@ -22773,14 +22773,14 @@
     <row r="493">
       <c r="A493" s="3" t="inlineStr">
         <is>
-          <t>new orleans matchmaker</t>
+          <t>malibu matchmaker</t>
         </is>
       </c>
       <c r="B493" s="4" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C493" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D493" s="10" t="inlineStr">
         <is>
@@ -22806,14 +22806,14 @@
     <row r="494">
       <c r="A494" s="3" t="inlineStr">
         <is>
-          <t>matchmaker salt lake city</t>
+          <t>newport beach matchmaker</t>
         </is>
       </c>
       <c r="B494" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C494" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D494" s="10" t="inlineStr">
         <is>
@@ -22839,14 +22839,14 @@
     <row r="495">
       <c r="A495" s="3" t="inlineStr">
         <is>
-          <t>naples matchmaker</t>
+          <t>matchmaker san jose</t>
         </is>
       </c>
       <c r="B495" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C495" s="2" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D495" s="10" t="inlineStr">
         <is>
@@ -22872,14 +22872,14 @@
     <row r="496">
       <c r="A496" s="3" t="inlineStr">
         <is>
-          <t>beverly hills matchmaker</t>
+          <t>palo alto matchmaker</t>
         </is>
       </c>
       <c r="B496" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="C496" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D496" s="10" t="inlineStr">
         <is>
@@ -22905,7 +22905,7 @@
     <row r="497">
       <c r="A497" s="3" t="inlineStr">
         <is>
-          <t>malibu matchmaker</t>
+          <t>atherton matchmaker</t>
         </is>
       </c>
       <c r="B497" s="4" t="n">
@@ -22938,7 +22938,7 @@
     <row r="498">
       <c r="A498" s="3" t="inlineStr">
         <is>
-          <t>newport beach matchmaker</t>
+          <t>hillsborough matchmaker</t>
         </is>
       </c>
       <c r="B498" s="4" t="n">
@@ -22971,14 +22971,14 @@
     <row r="499">
       <c r="A499" s="3" t="inlineStr">
         <is>
-          <t>matchmaker san jose</t>
+          <t>los altos matchmaker</t>
         </is>
       </c>
       <c r="B499" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C499" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D499" s="10" t="inlineStr">
         <is>
@@ -23004,7 +23004,7 @@
     <row r="500">
       <c r="A500" s="3" t="inlineStr">
         <is>
-          <t>palo alto matchmaker</t>
+          <t>scarsdale matchmaker</t>
         </is>
       </c>
       <c r="B500" s="4" t="n">
@@ -23037,7 +23037,7 @@
     <row r="501">
       <c r="A501" s="3" t="inlineStr">
         <is>
-          <t>atherton matchmaker</t>
+          <t>hamptons matchmaker</t>
         </is>
       </c>
       <c r="B501" s="4" t="n">
@@ -23070,7 +23070,7 @@
     <row r="502">
       <c r="A502" s="3" t="inlineStr">
         <is>
-          <t>hillsborough matchmaker</t>
+          <t>greenwich matchmaker</t>
         </is>
       </c>
       <c r="B502" s="4" t="n">
@@ -23103,7 +23103,7 @@
     <row r="503">
       <c r="A503" s="3" t="inlineStr">
         <is>
-          <t>los altos matchmaker</t>
+          <t>darien matchmaker</t>
         </is>
       </c>
       <c r="B503" s="4" t="n">
@@ -23136,7 +23136,7 @@
     <row r="504">
       <c r="A504" s="3" t="inlineStr">
         <is>
-          <t>scarsdale matchmaker</t>
+          <t>short hills matchmaker</t>
         </is>
       </c>
       <c r="B504" s="4" t="n">
@@ -23169,7 +23169,7 @@
     <row r="505">
       <c r="A505" s="3" t="inlineStr">
         <is>
-          <t>hamptons matchmaker</t>
+          <t>mclean matchmaker</t>
         </is>
       </c>
       <c r="B505" s="4" t="n">
@@ -23202,7 +23202,7 @@
     <row r="506">
       <c r="A506" s="3" t="inlineStr">
         <is>
-          <t>greenwich matchmaker</t>
+          <t>boca raton matchmaker</t>
         </is>
       </c>
       <c r="B506" s="4" t="n">
@@ -23235,7 +23235,7 @@
     <row r="507">
       <c r="A507" s="3" t="inlineStr">
         <is>
-          <t>darien matchmaker</t>
+          <t>park city matchmaker</t>
         </is>
       </c>
       <c r="B507" s="4" t="n">
@@ -23268,7 +23268,7 @@
     <row r="508">
       <c r="A508" s="3" t="inlineStr">
         <is>
-          <t>short hills matchmaker</t>
+          <t>highland park matchmaker</t>
         </is>
       </c>
       <c r="B508" s="4" t="n">
@@ -23301,7 +23301,7 @@
     <row r="509">
       <c r="A509" s="3" t="inlineStr">
         <is>
-          <t>mclean matchmaker</t>
+          <t>southlake matchmaker</t>
         </is>
       </c>
       <c r="B509" s="4" t="n">
@@ -23334,7 +23334,7 @@
     <row r="510">
       <c r="A510" s="3" t="inlineStr">
         <is>
-          <t>boca raton matchmaker</t>
+          <t>great falls matchmaker</t>
         </is>
       </c>
       <c r="B510" s="4" t="n">
@@ -23367,7 +23367,7 @@
     <row r="511">
       <c r="A511" s="3" t="inlineStr">
         <is>
-          <t>park city matchmaker</t>
+          <t>hinsdale matchmaker</t>
         </is>
       </c>
       <c r="B511" s="4" t="n">
@@ -23930,9 +23930,9 @@
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  120 articles, split exactly 40/40/40 across Months 1-3
-  36,870 total monthly searches addressed
+  36,700 total monthly searches addressed
   114 easy wins at KD &lt; 30 — front-loaded into Month 1 so you see local rankings early
-  Average difficulty KD 16.0 — deliberately achievable, weighted toward winnable local terms</t>
+  Average difficulty KD 16.3 — deliberately achievable, weighted toward winnable local terms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MM deck: year on best-of/review/cost titles (AEO recency)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>It's Just Lunch Reviews</t>
+          <t>It's Just Lunch Reviews (2026)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>How Much Does Tawkify Cost?</t>
+          <t>How Much Does Tawkify Cost in 2026?</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Luma Matchmaking: An Honest Review</t>
+          <t>Luma Matchmaking: An Honest Review (2026)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>How Much Does It's Just Lunch Cost?</t>
+          <t>How Much Does It's Just Lunch Cost in 2026?</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Three Day Rule Reviews</t>
+          <t>Three Day Rule Reviews (2026)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The Matchmaking Company Reviews</t>
+          <t>The Matchmaking Company Reviews (2026)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>The Best Alternatives to Dating Apps</t>
+          <t>The Best Alternatives to Dating Apps (2026)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>What Drives the Cost of Matchmaking Services</t>
+          <t>What Drives the Cost of Matchmaking Services (2026)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Selective Search: A Matchmaking Review</t>
+          <t>Selective Search: A Matchmaking Review (2026)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Best High-End Matchmaking Services</t>
+          <t>Best High-End Matchmaking Services (2026)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Best Elite Matchmaking Services</t>
+          <t>Best Elite Matchmaking Services (2026)</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Top Matchmaking Services, Compared</t>
+          <t>Top Matchmaking Services, Compared (2026)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Best Matchmakers in New York City</t>
+          <t>Best Matchmakers in New York City (2026)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Best Luxury Matchmaking Services</t>
+          <t>Best Luxury Matchmaking Services (2026)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kelleher International Reviews</t>
+          <t>Kelleher International Reviews (2026)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>How Much Does Three Day Rule Cost?</t>
+          <t>How Much Does Three Day Rule Cost in 2026?</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Professional Matchmaker Cost</t>
+          <t>Professional Matchmaker Cost (2026)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Los Angeles</t>
+          <t>Best Matchmakers in Los Angeles (2026)</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Florida</t>
+          <t>Best Matchmakers in Florida (2026)</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Miami</t>
+          <t>Best Matchmakers in Miami (2026)</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Chicago</t>
+          <t>Best Matchmakers in Chicago (2026)</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Dallas</t>
+          <t>Best Matchmakers in Dallas (2026)</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Washington, DC</t>
+          <t>Best Matchmakers in Washington, DC (2026)</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Atlanta</t>
+          <t>Best Matchmakers in Atlanta (2026)</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Best Matchmakers in Boston</t>
+          <t>Best Matchmakers in Boston (2026)</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Best Matchmakers in the San Francisco Bay Area</t>
+          <t>Best Matchmakers in the San Francisco Bay Area (2026)</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Best Matchmakers for Professionals</t>
+          <t>Best Matchmakers for Professionals (2026)</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Tawkify Alternatives Worth Considering</t>
+          <t>Tawkify Alternatives Worth Considering (2026)</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>It's Just Lunch Alternatives</t>
+          <t>It's Just Lunch Alternatives (2026)</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Tawkify vs It's Just Lunch</t>
+          <t>Tawkify vs It's Just Lunch (2026)</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>It's Just Lunch vs a High-Touch Matchmaker</t>
+          <t>It's Just Lunch vs a High-Touch Matchmaker (2026)</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Kelleher vs Selective Search: Elite Matchmaking Compared</t>
+          <t>Kelleher vs Selective Search: Elite Matchmaking Compared (2026)</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Elite Matchmaking Services, Compared</t>
+          <t>Elite Matchmaking Services, Compared (2026)</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Matchmaker Fees, Explained</t>
+          <t>Matchmaker Fees, Explained (2026)</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Matchmaking Service Prices: What You'll Pay</t>
+          <t>Matchmaking Service Prices: What You'll Pay (2026)</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>How Much Does a Personal Matchmaker Cost?</t>
+          <t>How Much Does a Personal Matchmaker Cost in 2026?</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>High-End Matchmaking: What the Price Includes</t>
+          <t>High-End Matchmaking: What the Price Includes (2026)</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Matchmaker Cost by Tier: Budget to Elite</t>
+          <t>Matchmaker Cost by Tier: Budget to Elite (2026)</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">

</xml_diff>

<commit_message>
MM deck: Reviews & Alternatives titles
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/master-matchmakers/keyword-research.xlsx
+++ b/decks/master-matchmakers/keyword-research.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Luma Matchmaking: An Honest Review (2026)</t>
+          <t>Luma Matchmaking Reviews &amp; Alternatives (2026)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Three Day Rule Reviews (2026)</t>
+          <t>Three Day Rule Reviews &amp; Alternatives (2026)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The Matchmaking Company Reviews (2026)</t>
+          <t>The Matchmaking Company Reviews &amp; Alternatives (2026)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Selective Search: A Matchmaking Review (2026)</t>
+          <t>Selective Search Reviews &amp; Alternatives (2026)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kelleher International Reviews (2026)</t>
+          <t>Kelleher International Reviews &amp; Alternatives (2026)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">

</xml_diff>